<commit_message>
Added missing data for large class of zulip project!
</commit_message>
<xml_diff>
--- a/util/Validation/ManualValidation/LazyClassForManual.xlsx
+++ b/util/Validation/ManualValidation/LazyClassForManual.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/neda/Desktop/workspace/BadSmells/util/Validation/ManualValidation/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{42C40C34-3DC9-2B40-A3D2-1A5A7A6DD264}" xr6:coauthVersionLast="46" xr6:coauthVersionMax="46" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5032A8CB-9AA8-C24A-BBEA-7667B0233C57}" xr6:coauthVersionLast="46" xr6:coauthVersionMax="46" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="26420" yWindow="1400" windowWidth="16280" windowHeight="15720" activeTab="1" xr2:uid="{572E1FC0-9749-4D45-A225-69C2C6421EF3}"/>
+    <workbookView xWindow="26420" yWindow="1400" windowWidth="16280" windowHeight="15720" xr2:uid="{572E1FC0-9749-4D45-A225-69C2C6421EF3}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -3202,7 +3202,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="5" spans="1:12" ht="17" hidden="1" thickTop="1" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:12" ht="17" thickTop="1" x14ac:dyDescent="0.2">
       <c r="A5" s="4" t="s">
         <v>15</v>
       </c>
@@ -3229,7 +3229,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="6" spans="1:12" ht="17" hidden="1" thickTop="1" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A6" s="4" t="s">
         <v>14</v>
       </c>
@@ -3256,7 +3256,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="7" spans="1:12" ht="17" hidden="1" thickTop="1" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A7" s="4" t="s">
         <v>16</v>
       </c>
@@ -3283,7 +3283,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="8" spans="1:12" ht="17" hidden="1" thickTop="1" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A8" s="4" t="s">
         <v>17</v>
       </c>
@@ -3310,7 +3310,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="9" spans="1:12" ht="17" hidden="1" thickTop="1" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A9" s="4" t="s">
         <v>847</v>
       </c>
@@ -3337,7 +3337,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="10" spans="1:12" ht="17" hidden="1" thickTop="1" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A10" s="4" t="s">
         <v>849</v>
       </c>
@@ -3364,7 +3364,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="11" spans="1:12" ht="17" hidden="1" thickTop="1" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A11" s="4" t="s">
         <v>18</v>
       </c>
@@ -3391,7 +3391,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="12" spans="1:12" ht="17" hidden="1" thickTop="1" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A12" s="4" t="s">
         <v>19</v>
       </c>
@@ -3418,7 +3418,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="13" spans="1:12" ht="17" hidden="1" thickTop="1" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A13" s="4" t="s">
         <v>20</v>
       </c>
@@ -3445,7 +3445,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="14" spans="1:12" ht="17" hidden="1" thickTop="1" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A14" s="4" t="s">
         <v>21</v>
       </c>
@@ -3472,7 +3472,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="15" spans="1:12" ht="17" hidden="1" thickTop="1" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A15" s="4" t="s">
         <v>22</v>
       </c>
@@ -3499,7 +3499,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="16" spans="1:12" ht="17" hidden="1" thickTop="1" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A16" s="4" t="s">
         <v>23</v>
       </c>
@@ -3526,7 +3526,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="17" spans="1:8" ht="17" hidden="1" thickTop="1" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A17" s="4" t="s">
         <v>24</v>
       </c>
@@ -3553,7 +3553,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="18" spans="1:8" ht="17" hidden="1" thickTop="1" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A18"/>
       <c r="G18" t="s">
         <v>6</v>
@@ -3562,7 +3562,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="19" spans="1:8" ht="17" hidden="1" thickTop="1" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A19"/>
       <c r="G19" t="s">
         <v>6</v>
@@ -3571,7 +3571,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="20" spans="1:8" ht="17" hidden="1" thickTop="1" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A20" s="4" t="s">
         <v>29</v>
       </c>
@@ -3598,7 +3598,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="21" spans="1:8" ht="17" hidden="1" thickTop="1" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A21" s="4" t="s">
         <v>30</v>
       </c>
@@ -3625,7 +3625,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="22" spans="1:8" ht="17" hidden="1" thickTop="1" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
         <v>32</v>
       </c>
@@ -3652,7 +3652,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="23" spans="1:8" ht="17" hidden="1" thickTop="1" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
         <v>34</v>
       </c>
@@ -3679,7 +3679,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="24" spans="1:8" ht="17" hidden="1" thickTop="1" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
         <v>35</v>
       </c>
@@ -3706,7 +3706,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="25" spans="1:8" ht="17" hidden="1" thickTop="1" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A25" s="4" t="s">
         <v>36</v>
       </c>
@@ -3733,7 +3733,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="26" spans="1:8" ht="17" hidden="1" thickTop="1" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A26" s="4" t="s">
         <v>37</v>
       </c>
@@ -3760,7 +3760,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="27" spans="1:8" ht="17" hidden="1" thickTop="1" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
         <v>38</v>
       </c>
@@ -3787,7 +3787,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="28" spans="1:8" ht="17" hidden="1" thickTop="1" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
         <v>39</v>
       </c>
@@ -3814,7 +3814,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="29" spans="1:8" ht="17" hidden="1" thickTop="1" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A29" s="4" t="s">
         <v>40</v>
       </c>
@@ -3841,7 +3841,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="30" spans="1:8" ht="17" hidden="1" thickTop="1" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A30" s="4" t="s">
         <v>41</v>
       </c>
@@ -3868,7 +3868,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="31" spans="1:8" ht="17" hidden="1" thickTop="1" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A31" s="4" t="s">
         <v>43</v>
       </c>
@@ -3895,7 +3895,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="32" spans="1:8" ht="17" hidden="1" thickTop="1" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A32" s="4" t="s">
         <v>44</v>
       </c>
@@ -3922,7 +3922,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="33" spans="1:8" ht="17" hidden="1" thickTop="1" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A33" s="4" t="s">
         <v>45</v>
       </c>
@@ -3949,7 +3949,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="34" spans="1:8" ht="17" hidden="1" thickTop="1" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A34" t="s">
         <v>46</v>
       </c>
@@ -3976,7 +3976,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="35" spans="1:8" ht="17" hidden="1" thickTop="1" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A35" s="4" t="s">
         <v>47</v>
       </c>
@@ -4003,7 +4003,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="36" spans="1:8" ht="17" hidden="1" thickTop="1" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A36" s="4" t="s">
         <v>48</v>
       </c>
@@ -4030,7 +4030,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="37" spans="1:8" ht="17" hidden="1" thickTop="1" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A37" s="4" t="s">
         <v>49</v>
       </c>
@@ -4057,7 +4057,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="38" spans="1:8" ht="17" hidden="1" thickTop="1" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A38" s="4" t="s">
         <v>50</v>
       </c>
@@ -4084,7 +4084,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="39" spans="1:8" ht="17" hidden="1" thickTop="1" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A39" s="4" t="s">
         <v>51</v>
       </c>
@@ -4111,7 +4111,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="40" spans="1:8" ht="17" hidden="1" thickTop="1" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A40" s="4" t="s">
         <v>52</v>
       </c>
@@ -4138,7 +4138,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="41" spans="1:8" ht="17" hidden="1" thickTop="1" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A41" t="s">
         <v>57</v>
       </c>
@@ -4165,7 +4165,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="42" spans="1:8" ht="17" hidden="1" thickTop="1" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A42" s="4" t="s">
         <v>851</v>
       </c>
@@ -4192,7 +4192,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="43" spans="1:8" ht="17" hidden="1" thickTop="1" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A43" s="4" t="s">
         <v>59</v>
       </c>
@@ -4219,7 +4219,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="44" spans="1:8" ht="17" thickTop="1" x14ac:dyDescent="0.2">
+    <row r="44" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A44" s="4" t="s">
         <v>60</v>
       </c>
@@ -4327,7 +4327,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="48" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="48" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A48" s="4" t="s">
         <v>65</v>
       </c>
@@ -4354,7 +4354,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="49" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="49" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A49" s="4" t="s">
         <v>66</v>
       </c>
@@ -4381,7 +4381,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="50" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="50" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A50" s="4" t="s">
         <v>67</v>
       </c>
@@ -4408,7 +4408,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="51" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="51" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A51" s="4" t="s">
         <v>68</v>
       </c>
@@ -4435,7 +4435,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="52" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="52" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A52" s="4" t="s">
         <v>69</v>
       </c>
@@ -4462,7 +4462,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="53" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="53" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A53" s="4" t="s">
         <v>70</v>
       </c>
@@ -4489,7 +4489,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="54" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="54" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A54" s="4" t="s">
         <v>71</v>
       </c>
@@ -4516,7 +4516,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="55" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="55" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A55" s="4" t="s">
         <v>73</v>
       </c>
@@ -4543,7 +4543,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="56" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="56" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A56" s="4" t="s">
         <v>74</v>
       </c>
@@ -4570,7 +4570,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="57" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="57" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A57" s="4" t="s">
         <v>76</v>
       </c>
@@ -4651,7 +4651,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="60" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="60" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A60" s="4" t="s">
         <v>80</v>
       </c>
@@ -4678,7 +4678,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="61" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="61" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A61" s="4" t="s">
         <v>81</v>
       </c>
@@ -4732,7 +4732,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="63" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="63" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A63" s="4" t="s">
         <v>84</v>
       </c>
@@ -4759,7 +4759,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="64" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="64" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A64" s="4" t="s">
         <v>852</v>
       </c>
@@ -4813,7 +4813,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="66" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="66" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A66" s="4" t="s">
         <v>86</v>
       </c>
@@ -4840,7 +4840,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="67" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="67" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A67" s="4" t="s">
         <v>88</v>
       </c>
@@ -4894,7 +4894,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="69" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="69" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A69" s="4" t="s">
         <v>91</v>
       </c>
@@ -4921,7 +4921,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="70" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="70" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A70" s="4" t="s">
         <v>92</v>
       </c>
@@ -4948,7 +4948,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="71" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="71" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A71" s="4" t="s">
         <v>93</v>
       </c>
@@ -4975,7 +4975,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="72" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="72" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A72" s="4" t="s">
         <v>94</v>
       </c>
@@ -5002,7 +5002,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="73" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="73" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A73" s="4" t="s">
         <v>95</v>
       </c>
@@ -5056,7 +5056,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="75" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="75" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A75" s="4" t="s">
         <v>97</v>
       </c>
@@ -5083,7 +5083,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="76" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="76" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A76" s="4" t="s">
         <v>98</v>
       </c>
@@ -5137,7 +5137,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="78" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="78" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A78" s="4" t="s">
         <v>102</v>
       </c>
@@ -5218,7 +5218,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="81" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="81" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A81" s="4" t="s">
         <v>105</v>
       </c>
@@ -5245,7 +5245,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="82" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="82" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A82" s="4" t="s">
         <v>106</v>
       </c>
@@ -5272,7 +5272,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="83" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="83" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A83" s="4" t="s">
         <v>107</v>
       </c>
@@ -5353,7 +5353,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="86" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="86" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A86" s="4" t="s">
         <v>112</v>
       </c>
@@ -5407,7 +5407,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="88" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="88" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A88" s="4" t="s">
         <v>115</v>
       </c>
@@ -5434,7 +5434,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="89" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="89" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A89" s="4" t="s">
         <v>117</v>
       </c>
@@ -5461,7 +5461,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="90" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="90" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A90" s="4" t="s">
         <v>118</v>
       </c>
@@ -5488,7 +5488,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="91" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="91" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A91" s="4" t="s">
         <v>119</v>
       </c>
@@ -5515,7 +5515,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="92" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="92" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A92" s="4" t="s">
         <v>120</v>
       </c>
@@ -5542,7 +5542,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="93" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="93" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A93" s="4" t="s">
         <v>121</v>
       </c>
@@ -5569,7 +5569,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="94" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="94" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A94" s="4" t="s">
         <v>122</v>
       </c>
@@ -5650,7 +5650,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="97" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="97" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A97" s="4" t="s">
         <v>126</v>
       </c>
@@ -5677,7 +5677,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="98" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="98" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A98" s="4" t="s">
         <v>853</v>
       </c>
@@ -5785,7 +5785,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="102" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="102" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A102" s="4" t="s">
         <v>130</v>
       </c>
@@ -5812,7 +5812,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="103" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="103" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A103" s="4" t="s">
         <v>131</v>
       </c>
@@ -5839,7 +5839,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="104" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="104" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A104" s="4" t="s">
         <v>132</v>
       </c>
@@ -5866,7 +5866,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="105" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="105" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A105" s="4" t="s">
         <v>133</v>
       </c>
@@ -5893,7 +5893,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="106" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="106" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A106" s="4" t="s">
         <v>134</v>
       </c>
@@ -5920,7 +5920,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="107" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="107" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A107" s="4" t="s">
         <v>55</v>
       </c>
@@ -5983,7 +5983,7 @@
         <v>139</v>
       </c>
     </row>
-    <row r="112" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="112" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A112" s="4" t="s">
         <v>141</v>
       </c>
@@ -6010,7 +6010,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="113" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="113" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A113" s="4" t="s">
         <v>142</v>
       </c>
@@ -6037,7 +6037,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="114" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="114" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A114" s="4" t="s">
         <v>143</v>
       </c>
@@ -6064,7 +6064,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="115" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="115" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A115" s="4" t="s">
         <v>144</v>
       </c>
@@ -6100,7 +6100,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="117" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="117" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A117" s="4" t="s">
         <v>147</v>
       </c>
@@ -6127,7 +6127,7 @@
         <v>146</v>
       </c>
     </row>
-    <row r="118" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="118" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A118" s="4" t="s">
         <v>148</v>
       </c>
@@ -6154,7 +6154,7 @@
         <v>146</v>
       </c>
     </row>
-    <row r="119" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="119" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A119" s="4" t="s">
         <v>149</v>
       </c>
@@ -6325,7 +6325,7 @@
         <v>165</v>
       </c>
     </row>
-    <row r="134" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="134" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A134" s="4" t="s">
         <v>167</v>
       </c>
@@ -6352,7 +6352,7 @@
         <v>166</v>
       </c>
     </row>
-    <row r="135" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="135" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A135" s="4" t="s">
         <v>168</v>
       </c>
@@ -6379,7 +6379,7 @@
         <v>166</v>
       </c>
     </row>
-    <row r="136" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="136" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A136" s="4" t="s">
         <v>169</v>
       </c>
@@ -6406,7 +6406,7 @@
         <v>166</v>
       </c>
     </row>
-    <row r="137" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="137" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A137" s="4" t="s">
         <v>171</v>
       </c>
@@ -6433,7 +6433,7 @@
         <v>170</v>
       </c>
     </row>
-    <row r="138" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="138" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A138" s="4" t="s">
         <v>848</v>
       </c>
@@ -6460,7 +6460,7 @@
         <v>172</v>
       </c>
     </row>
-    <row r="139" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="139" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A139" s="4" t="s">
         <v>850</v>
       </c>
@@ -6496,7 +6496,7 @@
         <v>173</v>
       </c>
     </row>
-    <row r="141" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="141" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A141" s="4" t="s">
         <v>175</v>
       </c>
@@ -6517,7 +6517,7 @@
         <v>174</v>
       </c>
     </row>
-    <row r="142" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="142" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A142" s="4" t="s">
         <v>176</v>
       </c>
@@ -6598,7 +6598,7 @@
         <v>181</v>
       </c>
     </row>
-    <row r="149" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="149" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A149" s="4" t="s">
         <v>183</v>
       </c>
@@ -6688,7 +6688,7 @@
         <v>190</v>
       </c>
     </row>
-    <row r="157" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="157" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A157" s="4" t="s">
         <v>192</v>
       </c>
@@ -6715,7 +6715,7 @@
         <v>191</v>
       </c>
     </row>
-    <row r="158" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="158" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A158" s="4" t="s">
         <v>193</v>
       </c>
@@ -6742,7 +6742,7 @@
         <v>191</v>
       </c>
     </row>
-    <row r="159" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="159" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A159" s="4" t="s">
         <v>194</v>
       </c>
@@ -6769,7 +6769,7 @@
         <v>191</v>
       </c>
     </row>
-    <row r="160" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="160" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A160" s="4" t="s">
         <v>195</v>
       </c>
@@ -6850,7 +6850,7 @@
         <v>191</v>
       </c>
     </row>
-    <row r="163" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="163" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A163" s="4" t="s">
         <v>198</v>
       </c>
@@ -6877,7 +6877,7 @@
         <v>191</v>
       </c>
     </row>
-    <row r="164" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="164" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A164" s="4" t="s">
         <v>199</v>
       </c>
@@ -6904,7 +6904,7 @@
         <v>191</v>
       </c>
     </row>
-    <row r="165" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="165" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A165" s="4" t="s">
         <v>200</v>
       </c>
@@ -6931,7 +6931,7 @@
         <v>191</v>
       </c>
     </row>
-    <row r="166" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="166" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A166" s="4" t="s">
         <v>202</v>
       </c>
@@ -6958,7 +6958,7 @@
         <v>201</v>
       </c>
     </row>
-    <row r="167" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="167" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A167" s="4" t="s">
         <v>203</v>
       </c>
@@ -6985,7 +6985,7 @@
         <v>201</v>
       </c>
     </row>
-    <row r="168" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="168" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A168" s="4" t="s">
         <v>207</v>
       </c>
@@ -7012,7 +7012,7 @@
         <v>201</v>
       </c>
     </row>
-    <row r="169" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="169" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A169" s="4" t="s">
         <v>204</v>
       </c>
@@ -7039,7 +7039,7 @@
         <v>201</v>
       </c>
     </row>
-    <row r="170" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="170" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A170" s="4" t="s">
         <v>205</v>
       </c>
@@ -7066,7 +7066,7 @@
         <v>201</v>
       </c>
     </row>
-    <row r="171" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="171" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A171" s="4" t="s">
         <v>206</v>
       </c>
@@ -7120,7 +7120,7 @@
         <v>210</v>
       </c>
     </row>
-    <row r="175" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="175" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A175" s="4" t="s">
         <v>212</v>
       </c>
@@ -7147,7 +7147,7 @@
         <v>211</v>
       </c>
     </row>
-    <row r="176" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="176" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A176" s="4" t="s">
         <v>213</v>
       </c>
@@ -7174,7 +7174,7 @@
         <v>211</v>
       </c>
     </row>
-    <row r="177" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="177" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A177" s="4" t="s">
         <v>215</v>
       </c>
@@ -7201,7 +7201,7 @@
         <v>214</v>
       </c>
     </row>
-    <row r="178" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="178" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A178" s="4" t="s">
         <v>216</v>
       </c>
@@ -7228,7 +7228,7 @@
         <v>214</v>
       </c>
     </row>
-    <row r="179" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="179" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A179" s="4" t="s">
         <v>217</v>
       </c>
@@ -7255,7 +7255,7 @@
         <v>214</v>
       </c>
     </row>
-    <row r="180" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="180" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A180" s="4" t="s">
         <v>218</v>
       </c>
@@ -7282,7 +7282,7 @@
         <v>214</v>
       </c>
     </row>
-    <row r="181" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="181" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A181" s="4" t="s">
         <v>219</v>
       </c>
@@ -7309,7 +7309,7 @@
         <v>214</v>
       </c>
     </row>
-    <row r="182" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="182" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A182" s="4" t="s">
         <v>220</v>
       </c>
@@ -7336,7 +7336,7 @@
         <v>214</v>
       </c>
     </row>
-    <row r="183" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="183" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A183" s="4" t="s">
         <v>221</v>
       </c>
@@ -7363,7 +7363,7 @@
         <v>214</v>
       </c>
     </row>
-    <row r="184" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="184" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A184" s="4" t="s">
         <v>222</v>
       </c>
@@ -7390,7 +7390,7 @@
         <v>214</v>
       </c>
     </row>
-    <row r="185" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="185" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A185" s="4" t="s">
         <v>223</v>
       </c>
@@ -7480,7 +7480,7 @@
         <v>229</v>
       </c>
     </row>
-    <row r="191" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="191" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A191" s="4" t="s">
         <v>231</v>
       </c>
@@ -7507,7 +7507,7 @@
         <v>230</v>
       </c>
     </row>
-    <row r="192" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="192" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A192" s="4" t="s">
         <v>232</v>
       </c>
@@ -7534,7 +7534,7 @@
         <v>230</v>
       </c>
     </row>
-    <row r="193" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="193" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A193" s="4" t="s">
         <v>233</v>
       </c>
@@ -7561,7 +7561,7 @@
         <v>230</v>
       </c>
     </row>
-    <row r="194" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="194" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A194" s="4" t="s">
         <v>235</v>
       </c>
@@ -7624,7 +7624,7 @@
         <v>238</v>
       </c>
     </row>
-    <row r="197" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="197" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A197" s="4" t="s">
         <v>240</v>
       </c>
@@ -7651,7 +7651,7 @@
         <v>239</v>
       </c>
     </row>
-    <row r="198" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="198" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A198" s="4" t="s">
         <v>242</v>
       </c>
@@ -7687,7 +7687,7 @@
         <v>243</v>
       </c>
     </row>
-    <row r="200" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="200" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A200" s="4" t="s">
         <v>245</v>
       </c>
@@ -7714,7 +7714,7 @@
         <v>244</v>
       </c>
     </row>
-    <row r="201" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="201" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A201" s="4" t="s">
         <v>246</v>
       </c>
@@ -7795,7 +7795,7 @@
         <v>244</v>
       </c>
     </row>
-    <row r="204" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="204" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A204" s="4" t="s">
         <v>250</v>
       </c>
@@ -7822,7 +7822,7 @@
         <v>249</v>
       </c>
     </row>
-    <row r="205" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="205" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A205" s="4" t="s">
         <v>252</v>
       </c>
@@ -7885,7 +7885,7 @@
         <v>256</v>
       </c>
     </row>
-    <row r="210" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="210" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A210" s="4" t="s">
         <v>258</v>
       </c>
@@ -7912,7 +7912,7 @@
         <v>257</v>
       </c>
     </row>
-    <row r="211" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="211" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A211" s="4" t="s">
         <v>259</v>
       </c>
@@ -7939,7 +7939,7 @@
         <v>257</v>
       </c>
     </row>
-    <row r="212" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="212" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A212" s="4" t="s">
         <v>260</v>
       </c>
@@ -7966,7 +7966,7 @@
         <v>257</v>
       </c>
     </row>
-    <row r="213" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="213" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A213" s="4" t="s">
         <v>261</v>
       </c>
@@ -7993,7 +7993,7 @@
         <v>257</v>
       </c>
     </row>
-    <row r="214" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="214" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A214" s="4" t="s">
         <v>262</v>
       </c>
@@ -8020,7 +8020,7 @@
         <v>257</v>
       </c>
     </row>
-    <row r="215" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="215" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A215" s="4" t="s">
         <v>263</v>
       </c>
@@ -8047,7 +8047,7 @@
         <v>257</v>
       </c>
     </row>
-    <row r="216" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="216" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A216" s="4" t="s">
         <v>264</v>
       </c>
@@ -8074,7 +8074,7 @@
         <v>257</v>
       </c>
     </row>
-    <row r="217" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="217" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A217" s="4" t="s">
         <v>265</v>
       </c>
@@ -8119,7 +8119,7 @@
         <v>267</v>
       </c>
     </row>
-    <row r="220" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="220" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A220" s="4" t="s">
         <v>269</v>
       </c>
@@ -8146,7 +8146,7 @@
         <v>268</v>
       </c>
     </row>
-    <row r="221" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="221" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A221" s="4" t="s">
         <v>270</v>
       </c>
@@ -8173,7 +8173,7 @@
         <v>268</v>
       </c>
     </row>
-    <row r="222" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="222" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A222" s="4" t="s">
         <v>271</v>
       </c>
@@ -8200,7 +8200,7 @@
         <v>268</v>
       </c>
     </row>
-    <row r="223" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="223" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A223" s="4" t="s">
         <v>85</v>
       </c>
@@ -8245,7 +8245,7 @@
         <v>273</v>
       </c>
     </row>
-    <row r="226" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="226" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A226" s="4" t="s">
         <v>275</v>
       </c>
@@ -8290,7 +8290,7 @@
         <v>277</v>
       </c>
     </row>
-    <row r="229" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="229" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A229" s="4" t="s">
         <v>279</v>
       </c>
@@ -8317,7 +8317,7 @@
         <v>278</v>
       </c>
     </row>
-    <row r="230" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="230" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A230" s="4" t="s">
         <v>280</v>
       </c>
@@ -8344,7 +8344,7 @@
         <v>278</v>
       </c>
     </row>
-    <row r="231" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="231" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A231" s="4" t="s">
         <v>281</v>
       </c>
@@ -8371,7 +8371,7 @@
         <v>278</v>
       </c>
     </row>
-    <row r="232" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="232" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A232" s="4" t="s">
         <v>283</v>
       </c>
@@ -8398,7 +8398,7 @@
         <v>282</v>
       </c>
     </row>
-    <row r="233" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="233" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A233" s="4" t="s">
         <v>284</v>
       </c>
@@ -8425,7 +8425,7 @@
         <v>282</v>
       </c>
     </row>
-    <row r="234" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="234" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A234" s="4" t="s">
         <v>285</v>
       </c>
@@ -8452,7 +8452,7 @@
         <v>282</v>
       </c>
     </row>
-    <row r="235" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="235" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A235" s="4" t="s">
         <v>286</v>
       </c>
@@ -8479,7 +8479,7 @@
         <v>282</v>
       </c>
     </row>
-    <row r="236" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="236" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A236" s="4" t="s">
         <v>287</v>
       </c>
@@ -8506,7 +8506,7 @@
         <v>282</v>
       </c>
     </row>
-    <row r="237" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="237" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A237" s="4" t="s">
         <v>288</v>
       </c>
@@ -8587,7 +8587,7 @@
         <v>291</v>
       </c>
     </row>
-    <row r="242" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="242" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A242" s="4" t="s">
         <v>293</v>
       </c>
@@ -8767,7 +8767,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="250" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="250" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A250" s="4" t="s">
         <v>303</v>
       </c>
@@ -8794,7 +8794,7 @@
         <v>302</v>
       </c>
     </row>
-    <row r="251" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="251" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A251" s="4" t="s">
         <v>304</v>
       </c>
@@ -8821,7 +8821,7 @@
         <v>302</v>
       </c>
     </row>
-    <row r="252" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="252" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A252" s="4" t="s">
         <v>305</v>
       </c>
@@ -8875,7 +8875,7 @@
         <v>302</v>
       </c>
     </row>
-    <row r="254" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="254" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A254" s="4" t="s">
         <v>308</v>
       </c>
@@ -8920,7 +8920,7 @@
         <v>310</v>
       </c>
     </row>
-    <row r="257" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="257" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A257" s="4" t="s">
         <v>312</v>
       </c>
@@ -8974,7 +8974,7 @@
         <v>313</v>
       </c>
     </row>
-    <row r="259" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="259" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A259" s="4" t="s">
         <v>315</v>
       </c>
@@ -9001,7 +9001,7 @@
         <v>318</v>
       </c>
     </row>
-    <row r="260" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="260" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A260" s="4" t="s">
         <v>316</v>
       </c>
@@ -9028,7 +9028,7 @@
         <v>318</v>
       </c>
     </row>
-    <row r="261" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="261" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A261" s="4" t="s">
         <v>320</v>
       </c>
@@ -9055,7 +9055,7 @@
         <v>317</v>
       </c>
     </row>
-    <row r="262" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="262" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A262" s="4" t="s">
         <v>321</v>
       </c>
@@ -9082,7 +9082,7 @@
         <v>319</v>
       </c>
     </row>
-    <row r="263" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="263" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A263" s="4" t="s">
         <v>323</v>
       </c>
@@ -9109,7 +9109,7 @@
         <v>322</v>
       </c>
     </row>
-    <row r="264" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="264" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A264" s="4" t="s">
         <v>324</v>
       </c>
@@ -9136,7 +9136,7 @@
         <v>322</v>
       </c>
     </row>
-    <row r="265" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="265" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A265" s="4" t="s">
         <v>325</v>
       </c>
@@ -9163,7 +9163,7 @@
         <v>322</v>
       </c>
     </row>
-    <row r="266" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="266" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A266" s="4" t="s">
         <v>326</v>
       </c>
@@ -9190,7 +9190,7 @@
         <v>322</v>
       </c>
     </row>
-    <row r="267" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="267" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A267" s="4" t="s">
         <v>328</v>
       </c>
@@ -9217,7 +9217,7 @@
         <v>327</v>
       </c>
     </row>
-    <row r="268" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="268" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A268" s="4" t="s">
         <v>330</v>
       </c>
@@ -9253,7 +9253,7 @@
         <v>331</v>
       </c>
     </row>
-    <row r="270" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="270" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A270" s="4" t="s">
         <v>333</v>
       </c>
@@ -9280,7 +9280,7 @@
         <v>332</v>
       </c>
     </row>
-    <row r="271" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="271" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A271" s="4" t="s">
         <v>334</v>
       </c>
@@ -9307,7 +9307,7 @@
         <v>332</v>
       </c>
     </row>
-    <row r="272" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="272" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A272" s="4" t="s">
         <v>335</v>
       </c>
@@ -9334,7 +9334,7 @@
         <v>332</v>
       </c>
     </row>
-    <row r="273" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="273" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A273" s="4" t="s">
         <v>336</v>
       </c>
@@ -9361,7 +9361,7 @@
         <v>332</v>
       </c>
     </row>
-    <row r="274" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="274" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A274" s="4" t="s">
         <v>337</v>
       </c>
@@ -9388,7 +9388,7 @@
         <v>332</v>
       </c>
     </row>
-    <row r="275" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="275" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A275" s="4" t="s">
         <v>338</v>
       </c>
@@ -9415,7 +9415,7 @@
         <v>332</v>
       </c>
     </row>
-    <row r="276" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="276" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A276" s="4" t="s">
         <v>339</v>
       </c>
@@ -9442,7 +9442,7 @@
         <v>332</v>
       </c>
     </row>
-    <row r="277" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="277" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A277" s="4" t="s">
         <v>340</v>
       </c>
@@ -9469,7 +9469,7 @@
         <v>332</v>
       </c>
     </row>
-    <row r="278" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="278" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A278" s="4" t="s">
         <v>341</v>
       </c>
@@ -9496,7 +9496,7 @@
         <v>332</v>
       </c>
     </row>
-    <row r="279" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="279" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A279" s="4" t="s">
         <v>342</v>
       </c>
@@ -9523,7 +9523,7 @@
         <v>332</v>
       </c>
     </row>
-    <row r="280" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="280" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A280" s="4" t="s">
         <v>343</v>
       </c>
@@ -9550,7 +9550,7 @@
         <v>332</v>
       </c>
     </row>
-    <row r="281" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="281" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A281" s="4" t="s">
         <v>344</v>
       </c>
@@ -9577,7 +9577,7 @@
         <v>332</v>
       </c>
     </row>
-    <row r="282" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="282" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A282" s="4" t="s">
         <v>345</v>
       </c>
@@ -9604,7 +9604,7 @@
         <v>332</v>
       </c>
     </row>
-    <row r="283" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="283" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A283" s="4" t="s">
         <v>346</v>
       </c>
@@ -9631,7 +9631,7 @@
         <v>332</v>
       </c>
     </row>
-    <row r="284" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="284" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A284" s="4" t="s">
         <v>347</v>
       </c>
@@ -9658,7 +9658,7 @@
         <v>332</v>
       </c>
     </row>
-    <row r="285" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="285" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A285" s="4" t="s">
         <v>348</v>
       </c>
@@ -9685,7 +9685,7 @@
         <v>332</v>
       </c>
     </row>
-    <row r="286" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="286" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A286" s="4" t="s">
         <v>349</v>
       </c>
@@ -9712,7 +9712,7 @@
         <v>332</v>
       </c>
     </row>
-    <row r="287" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="287" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A287" s="4" t="s">
         <v>350</v>
       </c>
@@ -9739,7 +9739,7 @@
         <v>332</v>
       </c>
     </row>
-    <row r="288" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="288" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A288" s="4" t="s">
         <v>351</v>
       </c>
@@ -9766,7 +9766,7 @@
         <v>332</v>
       </c>
     </row>
-    <row r="289" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="289" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A289" s="4" t="s">
         <v>352</v>
       </c>
@@ -9793,7 +9793,7 @@
         <v>332</v>
       </c>
     </row>
-    <row r="290" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="290" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A290" s="4" t="s">
         <v>353</v>
       </c>
@@ -9820,7 +9820,7 @@
         <v>332</v>
       </c>
     </row>
-    <row r="291" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="291" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A291" s="4" t="s">
         <v>354</v>
       </c>
@@ -9847,7 +9847,7 @@
         <v>332</v>
       </c>
     </row>
-    <row r="292" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="292" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A292" s="4" t="s">
         <v>355</v>
       </c>
@@ -9874,7 +9874,7 @@
         <v>332</v>
       </c>
     </row>
-    <row r="293" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="293" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A293" s="4" t="s">
         <v>356</v>
       </c>
@@ -9901,7 +9901,7 @@
         <v>332</v>
       </c>
     </row>
-    <row r="294" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="294" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A294" s="4" t="s">
         <v>357</v>
       </c>
@@ -9928,7 +9928,7 @@
         <v>332</v>
       </c>
     </row>
-    <row r="295" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="295" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A295" s="4" t="s">
         <v>358</v>
       </c>
@@ -9955,7 +9955,7 @@
         <v>332</v>
       </c>
     </row>
-    <row r="296" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="296" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A296" s="4" t="s">
         <v>359</v>
       </c>
@@ -9982,7 +9982,7 @@
         <v>332</v>
       </c>
     </row>
-    <row r="297" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="297" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A297" s="4" t="s">
         <v>360</v>
       </c>
@@ -10009,7 +10009,7 @@
         <v>332</v>
       </c>
     </row>
-    <row r="298" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="298" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A298" s="4" t="s">
         <v>361</v>
       </c>
@@ -10036,7 +10036,7 @@
         <v>332</v>
       </c>
     </row>
-    <row r="299" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="299" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A299" s="4" t="s">
         <v>362</v>
       </c>
@@ -10063,7 +10063,7 @@
         <v>332</v>
       </c>
     </row>
-    <row r="300" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="300" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A300" s="4" t="s">
         <v>363</v>
       </c>
@@ -10090,7 +10090,7 @@
         <v>332</v>
       </c>
     </row>
-    <row r="301" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="301" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A301" s="4" t="s">
         <v>364</v>
       </c>
@@ -10117,7 +10117,7 @@
         <v>332</v>
       </c>
     </row>
-    <row r="302" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="302" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A302" s="4" t="s">
         <v>365</v>
       </c>
@@ -10144,7 +10144,7 @@
         <v>332</v>
       </c>
     </row>
-    <row r="303" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="303" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A303" s="4" t="s">
         <v>367</v>
       </c>
@@ -10171,7 +10171,7 @@
         <v>332</v>
       </c>
     </row>
-    <row r="304" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="304" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A304" s="4" t="s">
         <v>368</v>
       </c>
@@ -10198,7 +10198,7 @@
         <v>332</v>
       </c>
     </row>
-    <row r="305" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="305" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A305" s="4" t="s">
         <v>369</v>
       </c>
@@ -10225,7 +10225,7 @@
         <v>332</v>
       </c>
     </row>
-    <row r="306" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="306" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A306" s="4" t="s">
         <v>366</v>
       </c>
@@ -10252,7 +10252,7 @@
         <v>332</v>
       </c>
     </row>
-    <row r="307" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="307" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A307" s="4" t="s">
         <v>370</v>
       </c>
@@ -10279,7 +10279,7 @@
         <v>332</v>
       </c>
     </row>
-    <row r="308" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="308" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A308" s="4" t="s">
         <v>371</v>
       </c>
@@ -10306,7 +10306,7 @@
         <v>332</v>
       </c>
     </row>
-    <row r="309" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="309" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A309" s="4" t="s">
         <v>372</v>
       </c>
@@ -10333,7 +10333,7 @@
         <v>332</v>
       </c>
     </row>
-    <row r="310" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="310" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A310" s="4" t="s">
         <v>373</v>
       </c>
@@ -10360,7 +10360,7 @@
         <v>332</v>
       </c>
     </row>
-    <row r="311" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="311" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A311" s="4" t="s">
         <v>374</v>
       </c>
@@ -10387,7 +10387,7 @@
         <v>332</v>
       </c>
     </row>
-    <row r="312" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="312" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A312" s="4" t="s">
         <v>375</v>
       </c>
@@ -10414,7 +10414,7 @@
         <v>332</v>
       </c>
     </row>
-    <row r="313" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="313" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A313" s="4" t="s">
         <v>384</v>
       </c>
@@ -10468,7 +10468,7 @@
         <v>332</v>
       </c>
     </row>
-    <row r="315" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="315" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A315" s="4" t="s">
         <v>386</v>
       </c>
@@ -10495,7 +10495,7 @@
         <v>332</v>
       </c>
     </row>
-    <row r="316" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="316" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A316" s="4" t="s">
         <v>376</v>
       </c>
@@ -10522,7 +10522,7 @@
         <v>332</v>
       </c>
     </row>
-    <row r="317" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="317" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A317" s="4" t="s">
         <v>387</v>
       </c>
@@ -10549,7 +10549,7 @@
         <v>332</v>
       </c>
     </row>
-    <row r="318" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="318" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A318" s="4" t="s">
         <v>388</v>
       </c>
@@ -10603,7 +10603,7 @@
         <v>332</v>
       </c>
     </row>
-    <row r="320" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="320" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A320" s="4" t="s">
         <v>377</v>
       </c>
@@ -10630,7 +10630,7 @@
         <v>332</v>
       </c>
     </row>
-    <row r="321" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="321" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A321" s="4" t="s">
         <v>390</v>
       </c>
@@ -10657,7 +10657,7 @@
         <v>332</v>
       </c>
     </row>
-    <row r="322" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="322" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A322" s="4" t="s">
         <v>391</v>
       </c>
@@ -10684,7 +10684,7 @@
         <v>332</v>
       </c>
     </row>
-    <row r="323" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="323" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A323" s="4" t="s">
         <v>392</v>
       </c>
@@ -10711,7 +10711,7 @@
         <v>332</v>
       </c>
     </row>
-    <row r="324" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="324" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A324" s="4" t="s">
         <v>378</v>
       </c>
@@ -10765,7 +10765,7 @@
         <v>332</v>
       </c>
     </row>
-    <row r="326" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="326" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A326" s="4" t="s">
         <v>380</v>
       </c>
@@ -10792,7 +10792,7 @@
         <v>332</v>
       </c>
     </row>
-    <row r="327" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="327" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A327" s="4" t="s">
         <v>393</v>
       </c>
@@ -10819,7 +10819,7 @@
         <v>332</v>
       </c>
     </row>
-    <row r="328" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="328" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A328" s="4" t="s">
         <v>381</v>
       </c>
@@ -10846,7 +10846,7 @@
         <v>332</v>
       </c>
     </row>
-    <row r="329" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="329" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A329" s="4" t="s">
         <v>394</v>
       </c>
@@ -10873,7 +10873,7 @@
         <v>332</v>
       </c>
     </row>
-    <row r="330" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="330" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A330" s="4" t="s">
         <v>395</v>
       </c>
@@ -10900,7 +10900,7 @@
         <v>332</v>
       </c>
     </row>
-    <row r="331" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="331" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A331" s="4" t="s">
         <v>396</v>
       </c>
@@ -10927,7 +10927,7 @@
         <v>332</v>
       </c>
     </row>
-    <row r="332" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="332" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A332" s="4" t="s">
         <v>397</v>
       </c>
@@ -10954,7 +10954,7 @@
         <v>332</v>
       </c>
     </row>
-    <row r="333" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="333" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A333" s="4" t="s">
         <v>398</v>
       </c>
@@ -10981,7 +10981,7 @@
         <v>332</v>
       </c>
     </row>
-    <row r="334" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="334" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A334" s="4" t="s">
         <v>399</v>
       </c>
@@ -11008,7 +11008,7 @@
         <v>332</v>
       </c>
     </row>
-    <row r="335" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="335" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A335" s="4" t="s">
         <v>400</v>
       </c>
@@ -11035,7 +11035,7 @@
         <v>332</v>
       </c>
     </row>
-    <row r="336" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="336" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A336" s="4" t="s">
         <v>401</v>
       </c>
@@ -11062,7 +11062,7 @@
         <v>332</v>
       </c>
     </row>
-    <row r="337" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="337" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A337" s="4" t="s">
         <v>382</v>
       </c>
@@ -11089,7 +11089,7 @@
         <v>332</v>
       </c>
     </row>
-    <row r="338" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="338" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A338" s="4" t="s">
         <v>402</v>
       </c>
@@ -11116,7 +11116,7 @@
         <v>332</v>
       </c>
     </row>
-    <row r="339" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="339" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A339" s="4" t="s">
         <v>403</v>
       </c>
@@ -11143,7 +11143,7 @@
         <v>332</v>
       </c>
     </row>
-    <row r="340" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="340" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A340" s="4" t="s">
         <v>404</v>
       </c>
@@ -11170,7 +11170,7 @@
         <v>332</v>
       </c>
     </row>
-    <row r="341" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="341" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A341" s="4" t="s">
         <v>405</v>
       </c>
@@ -11197,7 +11197,7 @@
         <v>332</v>
       </c>
     </row>
-    <row r="342" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="342" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A342" s="4" t="s">
         <v>406</v>
       </c>
@@ -11224,7 +11224,7 @@
         <v>332</v>
       </c>
     </row>
-    <row r="343" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="343" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A343" s="4" t="s">
         <v>407</v>
       </c>
@@ -11251,7 +11251,7 @@
         <v>332</v>
       </c>
     </row>
-    <row r="344" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="344" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A344" s="4" t="s">
         <v>408</v>
       </c>
@@ -11305,7 +11305,7 @@
         <v>332</v>
       </c>
     </row>
-    <row r="346" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="346" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A346" s="4" t="s">
         <v>409</v>
       </c>
@@ -11332,7 +11332,7 @@
         <v>332</v>
       </c>
     </row>
-    <row r="347" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="347" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A347" s="4" t="s">
         <v>410</v>
       </c>
@@ -11359,7 +11359,7 @@
         <v>332</v>
       </c>
     </row>
-    <row r="348" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="348" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A348" s="4" t="s">
         <v>411</v>
       </c>
@@ -11386,7 +11386,7 @@
         <v>332</v>
       </c>
     </row>
-    <row r="349" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="349" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A349" s="4" t="s">
         <v>412</v>
       </c>
@@ -11413,7 +11413,7 @@
         <v>332</v>
       </c>
     </row>
-    <row r="350" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="350" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A350" s="4" t="s">
         <v>413</v>
       </c>
@@ -11440,7 +11440,7 @@
         <v>332</v>
       </c>
     </row>
-    <row r="351" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="351" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A351" s="4" t="s">
         <v>414</v>
       </c>
@@ -11467,7 +11467,7 @@
         <v>332</v>
       </c>
     </row>
-    <row r="352" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="352" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A352" s="4" t="s">
         <v>415</v>
       </c>
@@ -11494,7 +11494,7 @@
         <v>332</v>
       </c>
     </row>
-    <row r="353" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="353" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A353" s="4" t="s">
         <v>416</v>
       </c>
@@ -11521,7 +11521,7 @@
         <v>332</v>
       </c>
     </row>
-    <row r="354" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="354" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A354" s="4" t="s">
         <v>417</v>
       </c>
@@ -11548,7 +11548,7 @@
         <v>332</v>
       </c>
     </row>
-    <row r="355" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="355" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A355" s="4" t="s">
         <v>418</v>
       </c>
@@ -11575,7 +11575,7 @@
         <v>332</v>
       </c>
     </row>
-    <row r="356" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="356" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A356" s="4" t="s">
         <v>419</v>
       </c>
@@ -11602,7 +11602,7 @@
         <v>332</v>
       </c>
     </row>
-    <row r="357" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="357" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A357" s="4" t="s">
         <v>420</v>
       </c>
@@ -11656,7 +11656,7 @@
         <v>423</v>
       </c>
     </row>
-    <row r="361" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="361" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A361" s="4" t="s">
         <v>425</v>
       </c>
@@ -11737,7 +11737,7 @@
         <v>427</v>
       </c>
     </row>
-    <row r="364" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="364" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A364" s="4" t="s">
         <v>429</v>
       </c>
@@ -11764,7 +11764,7 @@
         <v>428</v>
       </c>
     </row>
-    <row r="365" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="365" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A365" s="4" t="s">
         <v>431</v>
       </c>
@@ -11872,7 +11872,7 @@
         <v>436</v>
       </c>
     </row>
-    <row r="369" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="369" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A369" s="4" t="s">
         <v>438</v>
       </c>
@@ -11926,7 +11926,7 @@
         <v>439</v>
       </c>
     </row>
-    <row r="371" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="371" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A371" s="4" t="s">
         <v>441</v>
       </c>
@@ -11953,7 +11953,7 @@
         <v>439</v>
       </c>
     </row>
-    <row r="372" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="372" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A372" s="4" t="s">
         <v>443</v>
       </c>
@@ -11980,7 +11980,7 @@
         <v>442</v>
       </c>
     </row>
-    <row r="373" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="373" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A373" s="4" t="s">
         <v>445</v>
       </c>
@@ -12007,7 +12007,7 @@
         <v>444</v>
       </c>
     </row>
-    <row r="374" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="374" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A374" s="4" t="s">
         <v>447</v>
       </c>
@@ -12034,7 +12034,7 @@
         <v>446</v>
       </c>
     </row>
-    <row r="375" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="375" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A375" s="4" t="s">
         <v>449</v>
       </c>
@@ -12061,7 +12061,7 @@
         <v>448</v>
       </c>
     </row>
-    <row r="376" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="376" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A376" s="4" t="s">
         <v>451</v>
       </c>
@@ -12115,7 +12115,7 @@
         <v>452</v>
       </c>
     </row>
-    <row r="378" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="378" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A378" s="4" t="s">
         <v>455</v>
       </c>
@@ -12142,7 +12142,7 @@
         <v>454</v>
       </c>
     </row>
-    <row r="379" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="379" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A379" s="4" t="s">
         <v>457</v>
       </c>
@@ -12250,7 +12250,7 @@
         <v>462</v>
       </c>
     </row>
-    <row r="383" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="383" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A383" s="4" t="s">
         <v>464</v>
       </c>
@@ -12277,7 +12277,7 @@
         <v>462</v>
       </c>
     </row>
-    <row r="384" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="384" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A384" s="4" t="s">
         <v>466</v>
       </c>
@@ -12304,7 +12304,7 @@
         <v>465</v>
       </c>
     </row>
-    <row r="385" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="385" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A385" s="4" t="s">
         <v>468</v>
       </c>
@@ -12331,7 +12331,7 @@
         <v>467</v>
       </c>
     </row>
-    <row r="386" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="386" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A386" s="4" t="s">
         <v>470</v>
       </c>
@@ -12466,7 +12466,7 @@
         <v>477</v>
       </c>
     </row>
-    <row r="391" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="391" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A391" s="4" t="s">
         <v>479</v>
       </c>
@@ -12520,7 +12520,7 @@
         <v>478</v>
       </c>
     </row>
-    <row r="393" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="393" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A393" s="4" t="s">
         <v>481</v>
       </c>
@@ -12547,7 +12547,7 @@
         <v>478</v>
       </c>
     </row>
-    <row r="394" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="394" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A394" s="4" t="s">
         <v>482</v>
       </c>
@@ -12601,7 +12601,7 @@
         <v>478</v>
       </c>
     </row>
-    <row r="396" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="396" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A396" s="4" t="s">
         <v>484</v>
       </c>
@@ -12628,7 +12628,7 @@
         <v>478</v>
       </c>
     </row>
-    <row r="397" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="397" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A397" s="4" t="s">
         <v>485</v>
       </c>
@@ -12655,7 +12655,7 @@
         <v>478</v>
       </c>
     </row>
-    <row r="398" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="398" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A398" s="4" t="s">
         <v>487</v>
       </c>
@@ -12709,7 +12709,7 @@
         <v>488</v>
       </c>
     </row>
-    <row r="400" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="400" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A400" s="4" t="s">
         <v>491</v>
       </c>
@@ -12736,7 +12736,7 @@
         <v>490</v>
       </c>
     </row>
-    <row r="401" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="401" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A401" s="4" t="s">
         <v>492</v>
       </c>
@@ -12763,7 +12763,7 @@
         <v>490</v>
       </c>
     </row>
-    <row r="402" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="402" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A402" s="4" t="s">
         <v>493</v>
       </c>
@@ -12790,7 +12790,7 @@
         <v>490</v>
       </c>
     </row>
-    <row r="403" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="403" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A403" s="4" t="s">
         <v>495</v>
       </c>
@@ -12844,7 +12844,7 @@
         <v>496</v>
       </c>
     </row>
-    <row r="405" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="405" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A405" s="4" t="s">
         <v>499</v>
       </c>
@@ -12952,7 +12952,7 @@
         <v>503</v>
       </c>
     </row>
-    <row r="409" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="409" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A409" s="4" t="s">
         <v>506</v>
       </c>
@@ -13033,7 +13033,7 @@
         <v>512</v>
       </c>
     </row>
-    <row r="416" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="416" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A416" s="4" t="s">
         <v>514</v>
       </c>
@@ -13060,7 +13060,7 @@
         <v>513</v>
       </c>
     </row>
-    <row r="417" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="417" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A417" s="4" t="s">
         <v>515</v>
       </c>
@@ -13204,7 +13204,7 @@
         <v>527</v>
       </c>
     </row>
-    <row r="431" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="431" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A431" s="4" t="s">
         <v>529</v>
       </c>
@@ -13276,7 +13276,7 @@
         <v>534</v>
       </c>
     </row>
-    <row r="437" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="437" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A437" s="4" t="s">
         <v>536</v>
       </c>
@@ -13303,7 +13303,7 @@
         <v>535</v>
       </c>
     </row>
-    <row r="438" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="438" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A438" s="4" t="s">
         <v>537</v>
       </c>
@@ -13357,7 +13357,7 @@
         <v>535</v>
       </c>
     </row>
-    <row r="440" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="440" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A440" s="4" t="s">
         <v>540</v>
       </c>
@@ -13402,7 +13402,7 @@
         <v>542</v>
       </c>
     </row>
-    <row r="443" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="443" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A443" s="4" t="s">
         <v>544</v>
       </c>
@@ -13438,7 +13438,7 @@
         <v>545</v>
       </c>
     </row>
-    <row r="445" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="445" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A445" s="4" t="s">
         <v>547</v>
       </c>
@@ -13474,7 +13474,7 @@
         <v>548</v>
       </c>
     </row>
-    <row r="447" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="447" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A447" s="4" t="s">
         <v>550</v>
       </c>
@@ -13501,7 +13501,7 @@
         <v>549</v>
       </c>
     </row>
-    <row r="448" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="448" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A448" s="4" t="s">
         <v>551</v>
       </c>
@@ -13528,7 +13528,7 @@
         <v>549</v>
       </c>
     </row>
-    <row r="449" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="449" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A449" s="4" t="s">
         <v>552</v>
       </c>
@@ -13555,7 +13555,7 @@
         <v>549</v>
       </c>
     </row>
-    <row r="450" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="450" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A450" s="4" t="s">
         <v>553</v>
       </c>
@@ -13582,7 +13582,7 @@
         <v>549</v>
       </c>
     </row>
-    <row r="451" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="451" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A451" s="4" t="s">
         <v>554</v>
       </c>
@@ -13609,7 +13609,7 @@
         <v>549</v>
       </c>
     </row>
-    <row r="452" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="452" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A452" s="4" t="s">
         <v>555</v>
       </c>
@@ -13636,7 +13636,7 @@
         <v>549</v>
       </c>
     </row>
-    <row r="453" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="453" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A453" s="4" t="s">
         <v>556</v>
       </c>
@@ -13663,7 +13663,7 @@
         <v>549</v>
       </c>
     </row>
-    <row r="454" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="454" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A454" s="4" t="s">
         <v>557</v>
       </c>
@@ -13690,7 +13690,7 @@
         <v>549</v>
       </c>
     </row>
-    <row r="455" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="455" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A455" s="4" t="s">
         <v>558</v>
       </c>
@@ -13717,7 +13717,7 @@
         <v>549</v>
       </c>
     </row>
-    <row r="456" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="456" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A456" s="4" t="s">
         <v>560</v>
       </c>
@@ -13753,7 +13753,7 @@
         <v>561</v>
       </c>
     </row>
-    <row r="458" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="458" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A458" s="4" t="s">
         <v>563</v>
       </c>
@@ -13807,7 +13807,7 @@
         <v>562</v>
       </c>
     </row>
-    <row r="460" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="460" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A460" s="4" t="s">
         <v>565</v>
       </c>
@@ -13834,7 +13834,7 @@
         <v>562</v>
       </c>
     </row>
-    <row r="461" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="461" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A461" s="4" t="s">
         <v>855</v>
       </c>
@@ -13861,7 +13861,7 @@
         <v>566</v>
       </c>
     </row>
-    <row r="462" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="462" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A462" s="4" t="s">
         <v>567</v>
       </c>
@@ -13924,7 +13924,7 @@
         <v>571</v>
       </c>
     </row>
-    <row r="467" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="467" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A467" s="4" t="s">
         <v>573</v>
       </c>
@@ -13978,7 +13978,7 @@
         <v>576</v>
       </c>
     </row>
-    <row r="471" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="471" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A471" s="4" t="s">
         <v>578</v>
       </c>
@@ -14005,7 +14005,7 @@
         <v>577</v>
       </c>
     </row>
-    <row r="472" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="472" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A472" s="4" t="s">
         <v>580</v>
       </c>
@@ -14041,7 +14041,7 @@
         <v>581</v>
       </c>
     </row>
-    <row r="474" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="474" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A474" s="4" t="s">
         <v>583</v>
       </c>
@@ -14068,7 +14068,7 @@
         <v>582</v>
       </c>
     </row>
-    <row r="475" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="475" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A475" s="4" t="s">
         <v>585</v>
       </c>
@@ -14095,7 +14095,7 @@
         <v>584</v>
       </c>
     </row>
-    <row r="476" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="476" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A476" s="4" t="s">
         <v>587</v>
       </c>
@@ -14122,7 +14122,7 @@
         <v>586</v>
       </c>
     </row>
-    <row r="477" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="477" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A477" s="4" t="s">
         <v>588</v>
       </c>
@@ -14149,7 +14149,7 @@
         <v>586</v>
       </c>
     </row>
-    <row r="478" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="478" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A478" s="4" t="s">
         <v>589</v>
       </c>
@@ -14176,7 +14176,7 @@
         <v>586</v>
       </c>
     </row>
-    <row r="479" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="479" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A479" s="4" t="s">
         <v>590</v>
       </c>
@@ -14203,7 +14203,7 @@
         <v>586</v>
       </c>
     </row>
-    <row r="480" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="480" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A480" s="4" t="s">
         <v>592</v>
       </c>
@@ -14230,7 +14230,7 @@
         <v>591</v>
       </c>
     </row>
-    <row r="481" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="481" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A481" s="4" t="s">
         <v>593</v>
       </c>
@@ -14257,7 +14257,7 @@
         <v>591</v>
       </c>
     </row>
-    <row r="482" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="482" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A482" s="4" t="s">
         <v>595</v>
       </c>
@@ -14284,7 +14284,7 @@
         <v>594</v>
       </c>
     </row>
-    <row r="483" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="483" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A483" s="4" t="s">
         <v>596</v>
       </c>
@@ -14311,7 +14311,7 @@
         <v>594</v>
       </c>
     </row>
-    <row r="484" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="484" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A484" s="4" t="s">
         <v>597</v>
       </c>
@@ -14338,7 +14338,7 @@
         <v>594</v>
       </c>
     </row>
-    <row r="485" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="485" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A485" s="4" t="s">
         <v>598</v>
       </c>
@@ -14365,7 +14365,7 @@
         <v>594</v>
       </c>
     </row>
-    <row r="486" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="486" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A486" s="4" t="s">
         <v>599</v>
       </c>
@@ -14410,7 +14410,7 @@
         <v>601</v>
       </c>
     </row>
-    <row r="489" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="489" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A489" s="4" t="s">
         <v>603</v>
       </c>
@@ -14437,7 +14437,7 @@
         <v>602</v>
       </c>
     </row>
-    <row r="490" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="490" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A490" s="4" t="s">
         <v>604</v>
       </c>
@@ -14464,7 +14464,7 @@
         <v>602</v>
       </c>
     </row>
-    <row r="491" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="491" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A491" s="4" t="s">
         <v>605</v>
       </c>
@@ -14491,7 +14491,7 @@
         <v>602</v>
       </c>
     </row>
-    <row r="492" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="492" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A492" s="4" t="s">
         <v>606</v>
       </c>
@@ -14518,7 +14518,7 @@
         <v>602</v>
       </c>
     </row>
-    <row r="493" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="493" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A493" s="4" t="s">
         <v>607</v>
       </c>
@@ -14545,7 +14545,7 @@
         <v>602</v>
       </c>
     </row>
-    <row r="494" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="494" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A494" s="4" t="s">
         <v>608</v>
       </c>
@@ -14572,7 +14572,7 @@
         <v>602</v>
       </c>
     </row>
-    <row r="495" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="495" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A495" s="4" t="s">
         <v>609</v>
       </c>
@@ -14599,7 +14599,7 @@
         <v>602</v>
       </c>
     </row>
-    <row r="496" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="496" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A496" s="4" t="s">
         <v>610</v>
       </c>
@@ -14626,7 +14626,7 @@
         <v>602</v>
       </c>
     </row>
-    <row r="497" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="497" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A497" s="4" t="s">
         <v>611</v>
       </c>
@@ -14653,7 +14653,7 @@
         <v>602</v>
       </c>
     </row>
-    <row r="498" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="498" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A498" s="4" t="s">
         <v>612</v>
       </c>
@@ -14707,7 +14707,7 @@
         <v>602</v>
       </c>
     </row>
-    <row r="500" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="500" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A500" s="4" t="s">
         <v>614</v>
       </c>
@@ -14734,7 +14734,7 @@
         <v>602</v>
       </c>
     </row>
-    <row r="501" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="501" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A501" s="4" t="s">
         <v>615</v>
       </c>
@@ -14761,7 +14761,7 @@
         <v>602</v>
       </c>
     </row>
-    <row r="502" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="502" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A502" s="4" t="s">
         <v>616</v>
       </c>
@@ -14869,7 +14869,7 @@
         <v>602</v>
       </c>
     </row>
-    <row r="506" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="506" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A506" s="4" t="s">
         <v>620</v>
       </c>
@@ -14896,7 +14896,7 @@
         <v>602</v>
       </c>
     </row>
-    <row r="507" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="507" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A507" s="4" t="s">
         <v>621</v>
       </c>
@@ -14923,7 +14923,7 @@
         <v>602</v>
       </c>
     </row>
-    <row r="508" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="508" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A508" s="4" t="s">
         <v>622</v>
       </c>
@@ -14950,7 +14950,7 @@
         <v>602</v>
       </c>
     </row>
-    <row r="509" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="509" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A509" s="4" t="s">
         <v>624</v>
       </c>
@@ -14977,7 +14977,7 @@
         <v>623</v>
       </c>
     </row>
-    <row r="510" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="510" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A510" s="4" t="s">
         <v>625</v>
       </c>
@@ -15004,7 +15004,7 @@
         <v>623</v>
       </c>
     </row>
-    <row r="511" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="511" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A511" s="4" t="s">
         <v>626</v>
       </c>
@@ -15031,7 +15031,7 @@
         <v>623</v>
       </c>
     </row>
-    <row r="512" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="512" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A512" s="4" t="s">
         <v>627</v>
       </c>
@@ -15058,7 +15058,7 @@
         <v>623</v>
       </c>
     </row>
-    <row r="513" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="513" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A513" s="4" t="s">
         <v>628</v>
       </c>
@@ -15085,7 +15085,7 @@
         <v>623</v>
       </c>
     </row>
-    <row r="514" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="514" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A514" s="4" t="s">
         <v>629</v>
       </c>
@@ -15112,7 +15112,7 @@
         <v>623</v>
       </c>
     </row>
-    <row r="515" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="515" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A515" s="4" t="s">
         <v>630</v>
       </c>
@@ -15184,7 +15184,7 @@
         <v>634</v>
       </c>
     </row>
-    <row r="519" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="519" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A519" s="4" t="s">
         <v>636</v>
       </c>
@@ -15292,7 +15292,7 @@
         <v>642</v>
       </c>
     </row>
-    <row r="525" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="525" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A525" s="4" t="s">
         <v>645</v>
       </c>
@@ -15319,7 +15319,7 @@
         <v>644</v>
       </c>
     </row>
-    <row r="526" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="526" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A526" s="4" t="s">
         <v>647</v>
       </c>
@@ -15346,7 +15346,7 @@
         <v>646</v>
       </c>
     </row>
-    <row r="527" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="527" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A527" s="4" t="s">
         <v>649</v>
       </c>
@@ -15373,7 +15373,7 @@
         <v>648</v>
       </c>
     </row>
-    <row r="528" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="528" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A528" s="4" t="s">
         <v>651</v>
       </c>
@@ -15400,7 +15400,7 @@
         <v>650</v>
       </c>
     </row>
-    <row r="529" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="529" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A529" s="4" t="s">
         <v>653</v>
       </c>
@@ -15427,7 +15427,7 @@
         <v>652</v>
       </c>
     </row>
-    <row r="530" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="530" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A530" s="4" t="s">
         <v>655</v>
       </c>
@@ -15454,7 +15454,7 @@
         <v>654</v>
       </c>
     </row>
-    <row r="531" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="531" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A531" s="4" t="s">
         <v>856</v>
       </c>
@@ -15481,7 +15481,7 @@
         <v>656</v>
       </c>
     </row>
-    <row r="532" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="532" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A532" s="4" t="s">
         <v>657</v>
       </c>
@@ -15508,7 +15508,7 @@
         <v>656</v>
       </c>
     </row>
-    <row r="533" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="533" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A533" s="4" t="s">
         <v>658</v>
       </c>
@@ -15535,7 +15535,7 @@
         <v>656</v>
       </c>
     </row>
-    <row r="534" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="534" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A534" s="4" t="s">
         <v>659</v>
       </c>
@@ -15652,7 +15652,7 @@
         <v>669</v>
       </c>
     </row>
-    <row r="545" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="545" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A545" s="4" t="s">
         <v>671</v>
       </c>
@@ -15715,7 +15715,7 @@
         <v>675</v>
       </c>
     </row>
-    <row r="550" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="550" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A550" s="4" t="s">
         <v>677</v>
       </c>
@@ -15742,7 +15742,7 @@
         <v>676</v>
       </c>
     </row>
-    <row r="551" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="551" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A551" s="4" t="s">
         <v>678</v>
       </c>
@@ -15769,7 +15769,7 @@
         <v>676</v>
       </c>
     </row>
-    <row r="552" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="552" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A552" s="4" t="s">
         <v>679</v>
       </c>
@@ -15823,7 +15823,7 @@
         <v>676</v>
       </c>
     </row>
-    <row r="554" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="554" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A554" s="4" t="s">
         <v>681</v>
       </c>
@@ -15850,7 +15850,7 @@
         <v>676</v>
       </c>
     </row>
-    <row r="555" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="555" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A555" s="4" t="s">
         <v>682</v>
       </c>
@@ -15877,7 +15877,7 @@
         <v>676</v>
       </c>
     </row>
-    <row r="556" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="556" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A556" s="4" t="s">
         <v>683</v>
       </c>
@@ -15904,7 +15904,7 @@
         <v>676</v>
       </c>
     </row>
-    <row r="557" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="557" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A557" s="4" t="s">
         <v>684</v>
       </c>
@@ -15931,7 +15931,7 @@
         <v>676</v>
       </c>
     </row>
-    <row r="558" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="558" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A558" s="4" t="s">
         <v>686</v>
       </c>
@@ -16012,7 +16012,7 @@
         <v>687</v>
       </c>
     </row>
-    <row r="561" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="561" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A561" s="4" t="s">
         <v>691</v>
       </c>
@@ -16039,7 +16039,7 @@
         <v>690</v>
       </c>
     </row>
-    <row r="562" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="562" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A562" s="4" t="s">
         <v>692</v>
       </c>
@@ -16066,7 +16066,7 @@
         <v>690</v>
       </c>
     </row>
-    <row r="563" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="563" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A563" s="4" t="s">
         <v>693</v>
       </c>
@@ -16093,7 +16093,7 @@
         <v>690</v>
       </c>
     </row>
-    <row r="564" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="564" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A564" s="4" t="s">
         <v>694</v>
       </c>
@@ -16120,7 +16120,7 @@
         <v>690</v>
       </c>
     </row>
-    <row r="565" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="565" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A565" s="4" t="s">
         <v>695</v>
       </c>
@@ -16147,7 +16147,7 @@
         <v>690</v>
       </c>
     </row>
-    <row r="566" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="566" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A566" s="4" t="s">
         <v>697</v>
       </c>
@@ -16174,7 +16174,7 @@
         <v>696</v>
       </c>
     </row>
-    <row r="567" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="567" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A567" s="4" t="s">
         <v>698</v>
       </c>
@@ -16201,7 +16201,7 @@
         <v>696</v>
       </c>
     </row>
-    <row r="568" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="568" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A568" s="4" t="s">
         <v>699</v>
       </c>
@@ -16228,7 +16228,7 @@
         <v>696</v>
       </c>
     </row>
-    <row r="569" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="569" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A569" s="4" t="s">
         <v>700</v>
       </c>
@@ -16255,7 +16255,7 @@
         <v>696</v>
       </c>
     </row>
-    <row r="570" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="570" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A570" s="4" t="s">
         <v>701</v>
       </c>
@@ -16282,7 +16282,7 @@
         <v>696</v>
       </c>
     </row>
-    <row r="571" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="571" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A571" s="4" t="s">
         <v>702</v>
       </c>
@@ -16309,7 +16309,7 @@
         <v>696</v>
       </c>
     </row>
-    <row r="572" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="572" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A572" s="4" t="s">
         <v>703</v>
       </c>
@@ -16336,7 +16336,7 @@
         <v>696</v>
       </c>
     </row>
-    <row r="573" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="573" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A573" s="4" t="s">
         <v>704</v>
       </c>
@@ -16363,7 +16363,7 @@
         <v>696</v>
       </c>
     </row>
-    <row r="574" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="574" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A574" s="4" t="s">
         <v>705</v>
       </c>
@@ -16399,7 +16399,7 @@
         <v>707</v>
       </c>
     </row>
-    <row r="576" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="576" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A576" s="4" t="s">
         <v>709</v>
       </c>
@@ -16453,7 +16453,7 @@
         <v>710</v>
       </c>
     </row>
-    <row r="578" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="578" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A578" s="4" t="s">
         <v>712</v>
       </c>
@@ -16507,7 +16507,7 @@
         <v>710</v>
       </c>
     </row>
-    <row r="580" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="580" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A580" s="4" t="s">
         <v>714</v>
       </c>
@@ -16588,7 +16588,7 @@
         <v>710</v>
       </c>
     </row>
-    <row r="583" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="583" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A583" s="4" t="s">
         <v>717</v>
       </c>
@@ -16669,7 +16669,7 @@
         <v>710</v>
       </c>
     </row>
-    <row r="586" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="586" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A586" s="4" t="s">
         <v>720</v>
       </c>
@@ -16696,7 +16696,7 @@
         <v>710</v>
       </c>
     </row>
-    <row r="587" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="587" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A587" s="4" t="s">
         <v>721</v>
       </c>
@@ -16723,7 +16723,7 @@
         <v>710</v>
       </c>
     </row>
-    <row r="588" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="588" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A588" s="4" t="s">
         <v>722</v>
       </c>
@@ -16777,7 +16777,7 @@
         <v>710</v>
       </c>
     </row>
-    <row r="590" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="590" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A590" s="4" t="s">
         <v>724</v>
       </c>
@@ -16804,7 +16804,7 @@
         <v>710</v>
       </c>
     </row>
-    <row r="591" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="591" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A591" s="4" t="s">
         <v>725</v>
       </c>
@@ -16831,7 +16831,7 @@
         <v>710</v>
       </c>
     </row>
-    <row r="592" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="592" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A592" s="4" t="s">
         <v>726</v>
       </c>
@@ -16885,7 +16885,7 @@
         <v>710</v>
       </c>
     </row>
-    <row r="594" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="594" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A594" s="4" t="s">
         <v>728</v>
       </c>
@@ -16912,7 +16912,7 @@
         <v>710</v>
       </c>
     </row>
-    <row r="595" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="595" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A595" s="4" t="s">
         <v>729</v>
       </c>
@@ -16939,7 +16939,7 @@
         <v>710</v>
       </c>
     </row>
-    <row r="596" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="596" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A596" s="4" t="s">
         <v>730</v>
       </c>
@@ -16966,7 +16966,7 @@
         <v>710</v>
       </c>
     </row>
-    <row r="597" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="597" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A597" s="4" t="s">
         <v>731</v>
       </c>
@@ -16993,7 +16993,7 @@
         <v>710</v>
       </c>
     </row>
-    <row r="598" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="598" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A598" s="4" t="s">
         <v>732</v>
       </c>
@@ -17029,7 +17029,7 @@
         <v>733</v>
       </c>
     </row>
-    <row r="600" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="600" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A600" s="4" t="s">
         <v>735</v>
       </c>
@@ -17056,7 +17056,7 @@
         <v>734</v>
       </c>
     </row>
-    <row r="601" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="601" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A601" s="4" t="s">
         <v>736</v>
       </c>
@@ -17083,7 +17083,7 @@
         <v>734</v>
       </c>
     </row>
-    <row r="602" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="602" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A602" s="4" t="s">
         <v>737</v>
       </c>
@@ -17146,7 +17146,7 @@
         <v>741</v>
       </c>
     </row>
-    <row r="607" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="607" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A607" s="4" t="s">
         <v>743</v>
       </c>
@@ -17200,7 +17200,7 @@
         <v>746</v>
       </c>
     </row>
-    <row r="611" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="611" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A611" s="4" t="s">
         <v>799</v>
       </c>
@@ -17272,7 +17272,7 @@
         <v>751</v>
       </c>
     </row>
-    <row r="617" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="617" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A617" s="4" t="s">
         <v>800</v>
       </c>
@@ -17299,7 +17299,7 @@
         <v>752</v>
       </c>
     </row>
-    <row r="618" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="618" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A618" s="4" t="s">
         <v>801</v>
       </c>
@@ -17335,7 +17335,7 @@
         <v>753</v>
       </c>
     </row>
-    <row r="620" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="620" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A620" s="4" t="s">
         <v>802</v>
       </c>
@@ -17425,7 +17425,7 @@
         <v>761</v>
       </c>
     </row>
-    <row r="628" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="628" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A628" s="4" t="s">
         <v>795</v>
       </c>
@@ -17452,7 +17452,7 @@
         <v>762</v>
       </c>
     </row>
-    <row r="629" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="629" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A629" s="4" t="s">
         <v>796</v>
       </c>
@@ -17479,7 +17479,7 @@
         <v>763</v>
       </c>
     </row>
-    <row r="630" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="630" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A630" s="4" t="s">
         <v>797</v>
       </c>
@@ -17506,7 +17506,7 @@
         <v>763</v>
       </c>
     </row>
-    <row r="631" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="631" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A631" s="4" t="s">
         <v>798</v>
       </c>
@@ -17569,7 +17569,7 @@
         <v>767</v>
       </c>
     </row>
-    <row r="636" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="636" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A636" s="4" t="s">
         <v>769</v>
       </c>
@@ -17596,7 +17596,7 @@
         <v>768</v>
       </c>
     </row>
-    <row r="637" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="637" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A637" s="4" t="s">
         <v>858</v>
       </c>
@@ -17623,7 +17623,7 @@
         <v>770</v>
       </c>
     </row>
-    <row r="638" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="638" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A638" s="4" t="s">
         <v>803</v>
       </c>
@@ -17650,7 +17650,7 @@
         <v>770</v>
       </c>
     </row>
-    <row r="639" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="639" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A639" s="4" t="s">
         <v>804</v>
       </c>
@@ -17713,7 +17713,7 @@
         <v>775</v>
       </c>
     </row>
-    <row r="644" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="644" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A644" s="4" t="s">
         <v>777</v>
       </c>
@@ -17812,7 +17812,7 @@
         <v>785</v>
       </c>
     </row>
-    <row r="653" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="653" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A653" s="4" t="s">
         <v>805</v>
       </c>
@@ -17848,7 +17848,7 @@
         <v>787</v>
       </c>
     </row>
-    <row r="655" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="655" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A655" s="4" t="s">
         <v>806</v>
       </c>
@@ -17893,7 +17893,7 @@
         <v>790</v>
       </c>
     </row>
-    <row r="658" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="658" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A658" s="4" t="s">
         <v>807</v>
       </c>
@@ -17920,7 +17920,7 @@
         <v>791</v>
       </c>
     </row>
-    <row r="659" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="659" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A659" s="4" t="s">
         <v>808</v>
       </c>
@@ -17947,7 +17947,7 @@
         <v>791</v>
       </c>
     </row>
-    <row r="660" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="660" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A660" s="4" t="s">
         <v>809</v>
       </c>
@@ -17974,7 +17974,7 @@
         <v>791</v>
       </c>
     </row>
-    <row r="661" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="661" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A661" s="4" t="s">
         <v>810</v>
       </c>
@@ -18019,7 +18019,7 @@
         <v>793</v>
       </c>
     </row>
-    <row r="664" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="664" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A664" s="4" t="s">
         <v>811</v>
       </c>
@@ -18046,7 +18046,7 @@
         <v>794</v>
       </c>
     </row>
-    <row r="665" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="665" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A665" s="4" t="s">
         <v>813</v>
       </c>
@@ -18073,7 +18073,7 @@
         <v>794</v>
       </c>
     </row>
-    <row r="666" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="666" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A666" s="4" t="s">
         <v>812</v>
       </c>
@@ -18100,7 +18100,7 @@
         <v>794</v>
       </c>
     </row>
-    <row r="667" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="667" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A667" s="4" t="s">
         <v>815</v>
       </c>
@@ -18154,7 +18154,7 @@
         <v>818</v>
       </c>
     </row>
-    <row r="671" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="671" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A671" s="4" t="s">
         <v>820</v>
       </c>
@@ -18298,7 +18298,7 @@
         <v>832</v>
       </c>
     </row>
-    <row r="685" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="685" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A685" s="4" t="s">
         <v>834</v>
       </c>
@@ -18325,7 +18325,7 @@
         <v>833</v>
       </c>
     </row>
-    <row r="686" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="686" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A686" s="4" t="s">
         <v>836</v>
       </c>
@@ -18361,7 +18361,7 @@
         <v>837</v>
       </c>
     </row>
-    <row r="688" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="688" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A688" s="4" t="s">
         <v>839</v>
       </c>
@@ -18415,7 +18415,7 @@
         <v>842</v>
       </c>
     </row>
-    <row r="692" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+    <row r="692" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A692" s="4" t="s">
         <v>844</v>
       </c>
@@ -18462,12 +18462,9 @@
     </row>
   </sheetData>
   <autoFilter ref="A1:H694" xr:uid="{21E7C098-7B9E-FA42-965E-E1F15430CE6F}">
-    <filterColumn colId="0">
+    <filterColumn colId="5">
       <filters>
-        <filter val="AddReduceSeparate"/>
-        <filter val="IndexingSeparate"/>
-        <filter val="param"/>
-        <filter val="parameterized"/>
+        <filter val="Yes"/>
       </filters>
     </filterColumn>
   </autoFilter>

</xml_diff>